<commit_message>
Product Maintenance document set v1.4 and workbooks v1.1; document register and decision log updated
FRS v1.4, Process and Storyboards, UX Design and Reports, Notifications and Outputs v1.4,
Interface Specification, Developer Specification, Data Dictionary, User Stories and How to
Read this Pack v1.0; RTM, Fit-Gap, CR Register, Effort Estimate, Requirements Collection
and Walkthrough Users v1.1.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -1706,7 +1706,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Open: BRD-03, BRD-06, BRD-02 to complete</t>
+          <t>Open: BRD-06, BRD-02 to complete (BRD-03 complete)</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>BRD-03, BRD-06, BRD-02</t>
+          <t>BRD-06, BRD-02</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>These BRDs have the FRS and the review workbooks; BPS, UXD, RNO, DSP, DDI, USR and the How to read note are to be issued.</t>
+          <t>These BRDs have the FRS and the review workbooks; BPS, UXD, RNO, DSP, DDI, USR and the How to read note are to be issued. BRD-03 was completed on 16 Oct 2026.</t>
         </is>
       </c>
       <c r="G22" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Renewal document set v1.3 and workbooks v1.1; document register and decision log updated
FRS, Process and Storyboards, UX Design and Reports, Notifications and Outputs v1.3;
Interface Specification, Developer Specification, Data Dictionary, User Stories and How to
Read this Pack v1.0; RTM, Fit-Gap, CR Register, Effort Estimate, Requirements Collection and
Walkthrough Users v1.1. The FRS v1.2, its highlighted copy and the v1.0 workbooks are removed.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Open: BRD-06, BRD-02 to complete (BRD-03 complete)</t>
+          <t>Open: BRD-02 to complete (BRD-03 and BRD-06 complete)</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>O-001</t>
+          <t>D-012</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -1728,49 +1728,49 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-06</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Number of named users</t>
+          <t>Renewal FRS numbering</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>NFR-CAP-01 states 1,344 named users; the User Access sizing uses 530.</t>
+          <t>BDOI's FRRN numbers are kept; duplicate and short numbers of BDOI's FRS are corrected (FRRN.004.05, 013.03, 013.04, 038.04, 026.01, 027.0x, 029.0x) and the CBG Motor rules of BDOI's Annexes D and E are stated apart as FRRN.009.02.</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>BDOI to confirm the figure; capacity targets follow.</t>
+          <t>FRS Renewal v1.3, section Changes from Version 1.2.</t>
         </is>
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open: BDOI confirmation</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>NFR</t>
+          <t>FRS BRD-06 v1.3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>O-002</t>
+          <t>D-013</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -1780,49 +1780,49 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>BRD-11</t>
+          <t>BRD-06</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Dormant users and UIDM-ISC</t>
+          <t>Renewal change requests</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>A dormant user deactivated in BIBS returns active if UIDM-ISC sends the account as active.</t>
+          <t>Four change requests stay open: CR-RN-005 budget, CR-RN-008 CBG Motor rules, CR-RN-015 placement turnaround (delivered, for approval or removal) and CR-RN-024 accessibility; the other candidates of register v1.0 are BRD items, OOTB or Integration scope.</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>UIDM-ISC disables the account on the notice.</t>
+          <t>CR Register BRD-06 v1.1.</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open: BDOI approval (Q-RN-11)</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>NFR section 5</t>
+          <t>CR Register</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>O-003</t>
+          <t>O-001</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -1837,17 +1837,17 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>BRD-11</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Integration rate limit</t>
+          <t>Number of named users</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>A full re-synchronisation (about 2,600 calls) takes about 9 minutes at 300 calls a minute.</t>
+          <t>NFR-CAP-01 states 1,344 named users; the User Access sizing uses 530.</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>Agree the limit with BDOI IT before the load test.</t>
+          <t>BDOI to confirm the figure; capacity targets follow.</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
@@ -1867,14 +1867,14 @@
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>NFR section 5</t>
+          <t>NFR</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>O-004</t>
+          <t>O-002</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-11</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Quantum-resistant network encryption</t>
+          <t>Dormant users and UIDM-ISC</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>ASR 1.8.6 is not met.</t>
+          <t>A dormant user deactivated in BIBS returns active if UIDM-ISC sends the account as active.</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>Plan with BDOI IT.</t>
+          <t>UIDM-ISC disables the account on the notice.</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
@@ -1926,7 +1926,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>O-005</t>
+          <t>O-003</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -1941,17 +1941,17 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-11</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Backups after ransomware</t>
+          <t>Integration rate limit</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Immutable or cross-account backup copies are not yet confirmed (ASR 1.7.10).</t>
+          <t>A full re-synchronisation (about 2,600 calls) takes about 9 minutes at 300 calls a minute.</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>Confirm with BDOI IT.</t>
+          <t>Agree the limit with BDOI IT before the load test.</t>
         </is>
       </c>
       <c r="I20" s="12" t="inlineStr">
@@ -1971,14 +1971,14 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>NFR-REC-03</t>
+          <t>NFR section 5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>O-006</t>
+          <t>O-004</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -1998,12 +1998,12 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>References to the NFR register</t>
+          <t>Quantum-resistant network encryption</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>The System Requirements Specification and the Test Strategy v1.0 name the NFR document v1.0 and its register.</t>
+          <t>ASR 1.8.6 is not met.</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>They refer to this NFR v2.0 at their next issue.</t>
+          <t>Plan with BDOI IT.</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
@@ -2023,74 +2023,178 @@
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>SRS, Test Strategy</t>
+          <t>NFR section 5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
+          <t>O-005</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Backups after ransomware</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Immutable or cross-account backup copies are not yet confirmed (ASR 1.7.10).</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Confirm with BDOI IT.</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>NFR-REC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>O-006</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>References to the NFR register</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>The System Requirements Specification and the Test Strategy v1.0 name the NFR document v1.0 and its register.</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>They refer to this NFR v2.0 at their next issue.</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>SRS, Test Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
           <t>O-007</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>16 Oct 2026</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Observation</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>BRD-06, BRD-02</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>BRD-02</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Packs to complete</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>These BRDs have the FRS and the review workbooks; BPS, UXD, RNO, DSP, DDI, USR and the How to read note are to be issued. BRD-03 was completed on 16 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>BRD-02 has the FRS and the review workbooks; BPS, UXD, RNO, DSP, DDI, USR and the How to read note are to be issued. BRD-03 and BRD-06 were completed on 16 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT</t>
         </is>
       </c>
-      <c r="H22" s="12" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>Issue with the reusable builders of BRD-11.</t>
         </is>
       </c>
-      <c r="I22" s="12" t="inlineStr">
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J22" s="12" t="inlineStr">
+      <c r="J24" s="12" t="inlineStr">
         <is>
           <t>Document Register</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J22"/>
+  <autoFilter ref="A4:J24"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J522">
+  <conditionalFormatting sqref="A5:J524">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C522" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C524" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Operations Cashiering document set v3.4 and workbooks v1.1; document register and decision log updated
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Open: BRD-02 to complete (BRD-03 and BRD-06 complete)</t>
+          <t>Closed: BRD-11, BRD-03, BRD-06 and BRD-02 complete</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -1822,7 +1822,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>O-001</t>
+          <t>D-014</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -1832,49 +1832,49 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Number of named users</t>
+          <t>Cashiering FRS numbering</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>NFR-CAP-01 states 1,344 named users; the User Access sizing uses 530.</t>
+          <t>BDOI's FRS.CSH numbers are kept; slips of BDOI's FRS v3.1 are corrected: FRS.OPS.001 and FRS.OPS.002.0x become FRS.CSH.01.01.01 and FRS.CSH.01.02.0x; spaces in numbers removed; FRS.CSH.02.02.09.10 to .19 become FRS.CSH.02.02.10 to .19 (taxes on ORs move to FRS.CSH.02.02.20); the duplicate FRS.CSH.03.01.05 (selection) becomes FRS.CSH.03.01.04.03 and the duplicate FRS.CSH.04.01.03 becomes FRS.CSH.04.01.04; the report layout of FRS.CSH.09.02 becomes BR-CSH-21.</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>BDOI to confirm the figure; capacity targets follow.</t>
+          <t>FRS Operations Cashiering v3.4, section Changes from Version 3.3.</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open: BDOI confirmation</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>NFR</t>
+          <t>FRS BRD-02 v3.4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>O-002</t>
+          <t>D-015</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -1884,49 +1884,49 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>BRD-11</t>
+          <t>BRD-02</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Dormant users and UIDM-ISC</t>
+          <t>Cashiering change requests</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>A dormant user deactivated in BIBS returns active if UIDM-ISC sends the account as active.</t>
+          <t>Two change requests stay open: CR-CSH-101 time rules (not delivered) and CR-CSH-102 e-mail copy of the notices (delivered, for approval or removal); D-CSH-01 and D-CSH-02 are BRD requirements.</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>UIDM-ISC disables the account on the notice.</t>
+          <t>CR Register BRD-02 v1.1.</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open: BDOI approval (Q-CSH-09)</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>NFR section 5</t>
+          <t>CR Register</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>O-003</t>
+          <t>O-001</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -1941,17 +1941,17 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>BRD-11</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Integration rate limit</t>
+          <t>Number of named users</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>A full re-synchronisation (about 2,600 calls) takes about 9 minutes at 300 calls a minute.</t>
+          <t>NFR-CAP-01 states 1,344 named users; the User Access sizing uses 530.</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>Agree the limit with BDOI IT before the load test.</t>
+          <t>BDOI to confirm the figure; capacity targets follow.</t>
         </is>
       </c>
       <c r="I20" s="12" t="inlineStr">
@@ -1971,14 +1971,14 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>NFR section 5</t>
+          <t>NFR</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>O-004</t>
+          <t>O-002</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -1993,17 +1993,17 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-11</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Quantum-resistant network encryption</t>
+          <t>Dormant users and UIDM-ISC</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>ASR 1.8.6 is not met.</t>
+          <t>A dormant user deactivated in BIBS returns active if UIDM-ISC sends the account as active.</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>Plan with BDOI IT.</t>
+          <t>UIDM-ISC disables the account on the notice.</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
@@ -2030,7 +2030,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>O-005</t>
+          <t>O-003</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -2045,17 +2045,17 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>BRD-11</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Backups after ransomware</t>
+          <t>Integration rate limit</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Immutable or cross-account backup copies are not yet confirmed (ASR 1.7.10).</t>
+          <t>A full re-synchronisation (about 2,600 calls) takes about 9 minutes at 300 calls a minute.</t>
         </is>
       </c>
       <c r="G22" s="12" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>Confirm with BDOI IT.</t>
+          <t>Agree the limit with BDOI IT before the load test.</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
@@ -2075,14 +2075,14 @@
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>NFR-REC-03</t>
+          <t>NFR section 5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>O-006</t>
+          <t>O-004</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
@@ -2102,12 +2102,12 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>References to the NFR register</t>
+          <t>Quantum-resistant network encryption</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>The System Requirements Specification and the Test Strategy v1.0 name the NFR document v1.0 and its register.</t>
+          <t>ASR 1.8.6 is not met.</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>They refer to this NFR v2.0 at their next issue.</t>
+          <t>Plan with BDOI IT.</t>
         </is>
       </c>
       <c r="I23" s="12" t="inlineStr">
@@ -2127,74 +2127,282 @@
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>SRS, Test Strategy</t>
+          <t>NFR section 5</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
+          <t>O-005</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Backups after ransomware</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Immutable or cross-account backup copies are not yet confirmed (ASR 1.7.10).</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Confirm with BDOI IT.</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>NFR-REC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>O-006</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>References to the NFR register</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>The System Requirements Specification and the Test Strategy v1.0 name the NFR document v1.0 and its register.</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>They refer to this NFR v2.0 at their next issue.</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>SRS, Test Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
           <t>O-007</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>16 Oct 2026</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>Observation</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>BRD-02</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>Packs to complete</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>BRD-02 has the FRS and the review workbooks; BPS, UXD, RNO, DSP, DDI, USR and the How to read note are to be issued. BRD-03 and BRD-06 were completed on 16 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>The BRD-02 pack is complete: FRS, BPS, UXD and RNO v3.4, ICD, DSP, DDI, USR and How to read v1.0, workbooks v1.1.</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
-        <is>
-          <t>Issue with the reusable builders of BRD-11.</t>
-        </is>
-      </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Document Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>O-008</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>BRD-02</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Cashiering decisions open</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Minimal balance 10.00 (BRD) against -1.00 to 1.00 (BDOI's FRS); MBS has no group profile to maintain the AR and OR forms; the Check Pick-up screen stays in the Cashier profile although CSHID.009 is removed; dashboard links to applications outside BIBS wait for BDOI's list.</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>BDOI answers Q-CSH-01, Q-CSH-06, Q-CSH-07, Q-CSH-08.</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J24" s="12" t="inlineStr">
-        <is>
-          <t>Document Register</t>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>FRS BRD-02 v3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>O-009</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>BRD-03</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>Permissions in the Developer Specification</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>A few operations of the BRD-03 Developer Specification v1.0 show the permission JOURNAL_VIEW where the service checks PRODUCT_VIEW or PKG_REPORT_VIEW (shared constant name read from another class).</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Corrected at the next issue of the BRD-03 Developer Specification.</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>DSP BRD-03 v1.0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J24"/>
+  <autoFilter ref="A4:J28"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J524">
+  <conditionalFormatting sqref="A5:J528">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C524" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
BRD-03 Developer Specification v1.1 with the permissions the services check; Renewal list screenshot recaptured; password history of ten in the ASR compliance note
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -2221,17 +2221,17 @@
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>They refer to this NFR v2.0 at their next issue.</t>
+          <t>The SRS, the Test Strategy and the traceability matrix v1.1 refer to this NFR v2.0 and its register.</t>
         </is>
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
         <is>
-          <t>SRS, Test Strategy</t>
+          <t>SRS, Test Strategy, RTM v1.1</t>
         </is>
       </c>
     </row>
@@ -2377,17 +2377,17 @@
       </c>
       <c r="H28" s="12" t="inlineStr">
         <is>
-          <t>Corrected at the next issue of the BRD-03 Developer Specification.</t>
+          <t>Corrected in the BRD-03 Developer Specification v1.1: every operation shows the permission its service checks.</t>
         </is>
       </c>
       <c r="I28" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J28" s="12" t="inlineStr">
         <is>
-          <t>DSP BRD-03 v1.0</t>
+          <t>DSP BRD-03 v1.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
End-to-End Conformance Register v1.1: walkthroughs re-run on a fresh SIT/UAT environment, BRD-02/03/06/11 measured on their re-baselined BDOI-template FRS, gaps G03, G07, G10, G12 and G13 closed, new gaps G14 to G16; document register and decision log updated
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2391,18 +2391,70 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>O-010</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>End-to-End Conformance Register v1.1</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Conformance re-measured on a fresh SIT/UAT environment after the fixes since version 1.0. BRD-02, BRD-03, BRD-06 and BRD-11 are counted on the requirements of their BDOI-template FRS (v3.4, v1.4, v1.3, v1.6; BRD-11 on the UIDM-ISC and Entra ID model, FRUM.009 and FRUM.011 withdrawn, FRUM.014 new); the other BRDs on their BIBS FRS. Gaps G03 (except TAX-SLS and the two FY2027 true-up reports), G07, G10, G12 and G13 closed with evidence.</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Register v1.1 issued; v1.0 superseded.</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J28"/>
+  <autoFilter ref="A4:J29"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J528">
+  <conditionalFormatting sqref="A5:J529">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C528" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C529" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Product Maintenance document set v1.5 and End-to-End Conformance Register v1.3
FRS, UX Design, Process and Storyboards and Reports v1.5 of BRD-03 with the insurer page
(FRPM.023.02) and the field-level change history (FRPM.021.03); Developer Specification v1.2,
Data Dictionary v1.1 (insurer contacts and bank accounts), User Stories v1.1 and review
workbooks v1.2; the superseded versions are removed. Conformance Register v1.3 closes gaps G04,
G05, G08 and G09 on the automated checks of the release, with the parts left for later recorded
on each gap; decision log entry O-014, document register and drop indexes updated.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2599,18 +2599,70 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>O-014</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>End-to-End Conformance Register v1.3: gaps G04, G05, G08 and G09</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Report subscriptions with run-time permission and data-scope checks (G04), field-level master data change log with maker and checker read per record by the Auditor (G05), the full insurer page with contacts, payment terms and remittance, bank accounts and linked products under maker-checker (G08) and the daily service-invoice batch per insurer with its delivery status and re-send (G09) are delivered and closed on the automated checks of the release. Remaining parts recorded on each gap: report run time and password protection, the programme-wide change log screen, Risk Participation (CRQ08) and the insurer accounts view, the merged batch file and file-transfer channel (CRQ18).</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Register v1.3 issued; v1.2 superseded. Product Maintenance FRS, UX Design, Process and Storyboards and Reports v1.5, Developer Specification v1.2, Data Dictionary v1.1, User Stories v1.1 and review workbooks v1.2 issued.</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J32"/>
+  <autoFilter ref="A4:J33"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J532">
+  <conditionalFormatting sqref="A5:J533">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C532" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C533" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Product Maintenance set v1.6, Customer Servicing Facility FRS and test plan v1.2, Conformance Register v1.4
BRD-03: FRS, UX Design, Process and Storyboards and Reports v1.6 with the Ledger
Accounts tab of the insurer page (FRPM.023.02) and the Master Data Change Log
(FRPM.021.03); Developer Specification v1.3, User Stories v1.2 and review
workbooks v1.3. BRD-09: FRS and test plan v1.2 aligned with the case management
delivered. Conformance Register v1.4: gap G01 closed, BRD-09 walkthrough steps
P2.1 to P2.12 pass on a fresh SIT/UAT environment, remaining parts of G04, G05,
G08 and G09 delivered. Decision log entry O-015, document register and drop
indexes updated; superseded versions removed.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2651,18 +2651,70 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>O-015</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>End-to-End Conformance Register v1.4: case management (G01) and the remaining parts of G04, G05, G08 and G09</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Case management of the Customer Service Facility is delivered and closed (G01): logging, routing to the fulfilment units, resolution, return and CSR action, supervision, notes, documents, follow-up cases, SLA check with breach notices, Case Dashboard, case reports and Case Routing; the BRD-9 walkthrough steps P2.1 to P2.12 pass on a fresh SIT/UAT environment. Also delivered: report subscriptions at a time of day, on the last working day and with relative periods (G04); the Master Data Change Log screen with export, and the change history limited to the reader's data scope (G05); the insurer's ledger accounts on the insurer page (G08); supplementary service-invoice batches with one merged PDF and a manifest (G09). Open: password protection of confidential reports, Risk Participation (CRQ08), the file-transfer channel (CRQ18), the full case lists of the addendum (CSQ19).</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>Register v1.4 issued; v1.3 superseded. Product Maintenance FRS, UX Design, Process and Storyboards and Reports v1.6, Developer Specification v1.3, User Stories v1.2 and review workbooks v1.3 issued; Customer Servicing Facility FRS and test plan v1.2 issued.</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J33"/>
+  <autoFilter ref="A4:J34"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J533">
+  <conditionalFormatting sqref="A5:J534">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C533" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C534" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Conformance Register v1.5, decision log entry O-016 and document register
Register v1.5: walkthrough-script steps of BRD-00, BRD-08, BRD-12 and BRD-13
run again on a fresh SIT/UAT environment (351 pass, none fail, 2 blocked by
the partner portal); gaps G06 and G11 closed; G02 recorded as waiting for
BDOI (Drop 2 scope, EBQ13, UIDM-ISC provisioning of external users);
requirement evidence refreshed from the full build. v1.4 removed. Decision
log entry O-016; document register and drop indexes updated.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2703,18 +2703,70 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>O-016</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>End-to-End Conformance Register v1.5: data scope of records addressed by id, G06 and G11 closed, walkthrough recipes corrected</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Every screen action that opens or changes one record checks that the record belongs to a company and branch of the user's data access, otherwise it is answered as not found. Delivered and closed: the Layout panel of the reports with the MIS fields catalogue (G06) and New Policy and Edit of Submitted Policies (G11); the case routing notice is copied to the account officer. Walkthrough recipes corrected where they did not follow the screens or the release: BRD-00 J1.3, BRD-08 P1.3, P3.1 and P3.3 (Drop 2 process, assumption A-EB-06), BRD-13 FR-DM-125.1 and .2 (compiled and checked outside BIBS by design). Run again on a fresh SIT/UAT environment: 351 steps pass, none fail, 2 blocked. Open and waiting for BDOI: the partner portal (G02: Drop 2 scope, EBQ13, UIDM-ISC provisioning).</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>Register v1.5 issued; v1.4 superseded. Product Maintenance UX Design v1.7 issued; v1.6 superseded.</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J34"/>
+  <autoFilter ref="A4:J35"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J534">
+  <conditionalFormatting sqref="A5:J535">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C534" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C535" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Remittance and Claims UX Design v1.1 with screenshots, packs v1.1 and Conformance Register v1.7
Screens of the running application captured on seed data for the delivered
Remittance and Claims screens and the insurer co-insurance tab. UX Design,
Reports Notifications and Outputs, Developer Specification and Data
Dictionary v1.1 issued in the Remittance and Claims packs; Product
Maintenance UX Design v1.8. The Remittance and Claims FRS items are assessed
and counted in Conformance Register v1.7, with walkthrough checks of the
new claims tabs and the worklist export. Decision Log O-023.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2830,12 +2830,12 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Reinsurance deferred to Phase 2; risk participation (CRQ08) deferred with it</t>
+          <t>Reinsurance deferred to Phase 2; co-insurance stays in scope</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>The client decided that reinsurance is deferred to Phase 2. The platform keeps its reinsurance functions (reinsurer and reinsurance broker parties, receipts from a reinsurer, reinsurance settlement payments) behind one permission that no BDOI group profile holds: the screens do not offer them and the server refuses them to the BDOI roles; the super user of DEV, SIT and UAT keeps them. The Data Migration console stays with the migration roles of the FRS and the super user and is not given to the business personas. Risk participation on the insurer record (CRQ08) is a reinsurance and co-insurance participation concept and is deferred with reinsurance; the co-insurance split of an invoice stays in Operations (FR-OP-007).</t>
+          <t>The client decided that reinsurance is deferred to Phase 2. The platform keeps its reinsurance functions (reinsurer and reinsurance broker parties, receipts from a reinsurer, reinsurance settlement payments) behind one permission that no BDOI group profile holds: the screens do not offer them and the server refuses them to the BDOI roles; the super user of DEV, SIT and UAT keeps them. The Data Migration console stays with the migration roles of the FRS and the super user and is not given to the business personas. Co-insurance is not deferred: the co-insurer parties, the co-insurance split of an invoice (FR-OP-007) and the default co-insurance participation on the insurer (CRQ08 Risk Participation) are in scope (corrected by O-022).</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>FRS BRD-00 v1.2 issued; gap G17 recorded as Deferred to Phase 2.</t>
+          <t>FRS BRD-00 v1.2 issued; gap G17 recorded as Deferred to Phase 2; corrected in FRS BRD-00 v1.3.</t>
         </is>
       </c>
       <c r="I37" s="12" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="J37" s="12" t="inlineStr">
         <is>
-          <t>FRS BRD-00 v1.2</t>
+          <t>FRS BRD-00 v1.3</t>
         </is>
       </c>
     </row>
@@ -3015,18 +3015,122 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>O-022</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>Co-insurance in scope; CRQ08 Risk Participation back in scope</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>The client confirmed that co-insurance is in scope of the current phase; only reinsurance is deferred to Phase 2. The earlier decision of 17-Oct-2026 had deferred CRQ08 Risk Participation with reinsurance because the BRD-00 FRS described it as default co-insurance shares on the insurer; that is reversed. Delivered: the Co-insurance / Risk Participation tab of the insurer page (participating insurers, share %, lead insurer flag, effective dates; maker-checker and the change log; shares of one period up to 100 %), used as the default co-insurance split of an invoice booked without one when the authorized shares in force total 100 % (FR-OP-007). Checked: the switch-off of the reinsurance functions hides only reinsurer and reinsurance-broker items; the co-insurer party type and the co-insurance functions stay open to the BDOI roles.</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Client (BDOI)</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>FRS BRD-00 v1.3 issued; O-018 corrected; gaps G08 and G17 restated.</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>FRS BRD-00 v1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>O-023</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>BRD-02, BRD-07</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>Remittance and Claims FRS in BDOI's format assessed and counted</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>The items of the Remittance FRS v1.0 and the Claims FRS v1.0, listed apart in register v1.6 as not yet assessed, are assessed and counted from register v1.7: BRD-02 against the Cashiering FRS v3.4 and the Remittance FRS v1.0, BRD-07 against the Claims FRS v1.0. Items delivered in the release of 17-Oct-2026 are conformant on the automated checks and the walkthrough steps; the others take the result of their fit-gap (Fit conformant, Partial partly conformant, Gap not conformant, change request not testable yet until BDOI approves it, integration partly conformant on the simulator). The two Remittance items specified in another FRS are not counted. The change requests CR-CLM-101 to 112 are not delivered. Current phase: 388 of 637 requirements conformant (60.9%), 212 partly, 37 not testable yet, none not conformant.</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.7 issued; v1.6 superseded. UX Design, Reports Notifications and Outputs, Developer Specification and Data Dictionary v1.1 issued in both packs with screenshots of the running application.</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J42" s="12" t="inlineStr">
+        <is>
+          <t>Conformance Register v1.7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J40"/>
+  <autoFilter ref="A4:J42"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J540">
+  <conditionalFormatting sqref="A5:J542">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C540" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C542" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
System Requirements Specification v1.2 with one chapter per BRD, SRS extracts and traceability matrix v1.2
The SRS is restructured into the common requirements and one chapter per
BRD; each system requirement is tagged with its BRD and traced to its FRS
(in BDOI's format for BRD-02, BRD-03, BRD-06, BRD-07 and BRD-11) and the
document reflects the deliveries and client decisions to 17-Oct-2026. A
5 to 10 page extract of each chapter is issued into the six packs and
listed in their How to Read notes. The traceability matrix v1.2 adds the
System requirements sheet. The Conformance Register v1.7 leaves out the
Remittance requirement specified in other FRS and uses Product Maintenance
FRS v1.7. Decision Log O-024; document register and indexes refreshed.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Common/BIBS_Log_BRD-00_Decision_and_Observation_Log_v1.0.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$4:$J$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>The items of the Remittance FRS v1.0 and the Claims FRS v1.0, listed apart in register v1.6 as not yet assessed, are assessed and counted from register v1.7: BRD-02 against the Cashiering FRS v3.4 and the Remittance FRS v1.0, BRD-07 against the Claims FRS v1.0. Items delivered in the release of 17-Oct-2026 are conformant on the automated checks and the walkthrough steps; the others take the result of their fit-gap (Fit conformant, Partial partly conformant, Gap not conformant, change request not testable yet until BDOI approves it, integration partly conformant on the simulator). The two Remittance items specified in another FRS are not counted. The change requests CR-CLM-101 to 112 are not delivered. Current phase: 388 of 637 requirements conformant (60.9%), 212 partly, 37 not testable yet, none not conformant.</t>
+          <t>The items of the Remittance FRS v1.0 and the Claims FRS v1.0, listed apart in register v1.6 as not yet assessed, are assessed and counted from register v1.7: BRD-02 against the Cashiering FRS v3.4 and the Remittance FRS v1.0, BRD-07 against the Claims FRS v1.0. Items delivered in the release of 17-Oct-2026 are conformant on the automated checks and the walkthrough steps; the others take the result of their fit-gap (Fit conformant, Partial partly conformant, Gap not conformant, change request not testable yet until BDOI approves it, integration partly conformant on the simulator). The two Remittance items specified in another FRS are not counted. The change requests CR-CLM-101 to 112 are not delivered. Current phase: 388 of 636 requirements conformant (61.0%), 212 partly, 36 not testable yet, none not conformant.</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
@@ -3119,18 +3119,70 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>O-024</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>BRD-00</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>System Requirements Specification v1.2: common requirements and one chapter per BRD</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>The SRS is restructured into the common requirements (BRD-00) and one chapter per BRD; each of its 643 system requirements is tagged with its BRD and traced to the IDs of its FRS (the FRS in BDOI's format for BRD-02, BRD-03, BRD-06, BRD-07 and BRD-11). It reflects the deliveries and client decisions to 17-Oct-2026: users and group profiles from UIDM-ISC with sign-in through Entra ID, case management of the Customer Servicing Facility, reinsurance and the partner portal in Phase 2 and co-insurance in the current phase. Each pack in BDOI's format carries the extract of its chapter and an access matrix.</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>SRS v1.2 and traceability matrix v1.2 (System requirements sheet) issued; v1.1 superseded. SRS extract v1.2 and Access Matrix v1.0 in the six packs.</t>
+        </is>
+      </c>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="J43" s="12" t="inlineStr">
+        <is>
+          <t>SRS v1.2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J42"/>
+  <autoFilter ref="A4:J43"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:J542">
+  <conditionalFormatting sqref="A5:J543">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C542" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="C5:C543" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>